<commit_message>
build: android, fix: fish
</commit_message>
<xml_diff>
--- a/Sheets/decor_catalog.xlsx
+++ b/Sheets/decor_catalog.xlsx
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=1a297ceb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=43252278")</f>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -2487,24 +2487,24 @@
     <row r="3" ht="66" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">blue-bee-betta</t>
+          <t xml:space="preserve">blue-flame-betta</t>
         </is>
       </c>
       <c r="B3" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-bee-betta.png?v=f43bfe73")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=9950f4a4")</f>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Ong Xanh</t>
+          <t xml:space="preserve">Blue Flame Betta</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đen xanh dương, khoang vàng · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Xanh dương, đỏ, cam · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E3" s="4">
-        <v>1400</v>
+        <v>900</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -2520,24 +2520,24 @@
     <row r="4" ht="66" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">blue-flame-betta</t>
+          <t xml:space="preserve">blue-panda-betta</t>
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=cdd432e5")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=1cbc3e15")</f>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Flame Betta</t>
+          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xanh dương, đỏ, cam · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Thân trắng hồng đốm đen, đuôi trắng mảng xanh dương đậm · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E4" s="4">
-        <v>900</v>
+        <v>1800</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
@@ -2553,24 +2553,24 @@
     <row r="5" ht="66" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">blue-panda-betta</t>
+          <t xml:space="preserve">blue-wild-betta</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=36b3bf65")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=e36e243b")</f>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
+          <t xml:space="preserve">Betta Rồng Xanh</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thân trắng hồng đốm đen, đuôi trắng mảng xanh dương đậm · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Betta hoang dã xanh lam, đốm đen trên vây · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E5" s="4">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -2586,24 +2586,24 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">blue-wild-betta</t>
+          <t xml:space="preserve">colorful-betta</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=680bdef4")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=5cc1541c")</f>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Rồng Xanh</t>
+          <t xml:space="preserve">Colorful Betta</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta hoang dã xanh lam, đốm đen trên vây · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Xanh dương, đỏ, trắng, vàng · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E6" s="4">
-        <v>2000</v>
+        <v>800</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
@@ -2619,24 +2619,24 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">colorful-betta</t>
+          <t xml:space="preserve">emerald-red-betta</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=b244d109")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/emerald-red-betta.png?v=c2d27f6b")</f>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colorful Betta</t>
+          <t xml:space="preserve">Betta Lục Bảo Đỏ</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xanh dương, đỏ, trắng, vàng · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Thân vảy xanh lục bảo, vây đỏ viền sẫm, đuôi bán nguyệt · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E7" s="4">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=c0b59211")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=ab617dcf")</f>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b4f93beb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b85cc880")</f>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=e769ef5b")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=798a58a8")</f>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=e1ab2904")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=f57fa2a7")</f>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=8fa1bfac")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=0a139958")</f>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=217c12a3")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=d3f82500")</f>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
@@ -2854,16 +2854,16 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=82c21339")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=a66df8df")</f>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plakat Galaxy</t>
+          <t xml:space="preserve">Koi Galaxy Betta</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Koi Galaxy: thân trắng ngọc mảng đỏ tươi, lưng vảy đen, mang trắng viền đỏ, vây vàng nghệ</t>
+          <t xml:space="preserve">Thân trắng ngọc mảng đỏ tươi, lưng vảy đen, mang trắng viền đỏ, vây vàng nghệ</t>
         </is>
       </c>
       <c r="E14" s="4">
@@ -2883,24 +2883,24 @@
     <row r="15" ht="66" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">purple-ruby-betta</t>
+          <t xml:space="preserve">purple-moon-betta</t>
         </is>
       </c>
       <c r="B15" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=dd6ba697")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-moon-betta.png?v=f988dcb3")</f>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
+          <t xml:space="preserve">Betta Trăng Tím</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thân tím hồng, đầu và vây đỏ hồng ngọc viền trắng · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Thân vảy bạc ánh kim, vây tím crôm, đuôi bán nguyệt viền trắng · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E15" s="4">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
@@ -2916,24 +2916,24 @@
     <row r="16" ht="66" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">red-steel-betta</t>
+          <t xml:space="preserve">purple-ruby-betta</t>
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=b64f1149")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=8b2a77a6")</f>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Steel Betta</t>
+          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thân xanh thép, vây đỏ trắng · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Thân tím hồng, đầu và vây đỏ hồng ngọc viền trắng · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E16" s="4">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
@@ -2949,24 +2949,24 @@
     <row r="17" ht="66" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">royal-koi-betta</t>
+          <t xml:space="preserve">red-steel-betta</t>
         </is>
       </c>
       <c r="B17" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=e1d369c0")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=e29f7895")</f>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Royal Koi</t>
+          <t xml:space="preserve">Red Steel Betta</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Koi xanh hoàng gia, đỏ, vàng · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Thân xanh thép, vây đỏ trắng · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E17" s="4">
-        <v>2200</v>
+        <v>900</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -2982,24 +2982,24 @@
     <row r="18" ht="66" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sky-koi-betta</t>
+          <t xml:space="preserve">royal-koi-betta</t>
         </is>
       </c>
       <c r="B18" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=b28bfda2")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=413784be")</f>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta</t>
+          <t xml:space="preserve">Royal Koi</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xanh da trời, đỏ, cam · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Koi xanh hoàng gia, đỏ, vàng · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E18" s="4">
-        <v>1000</v>
+        <v>2200</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
@@ -3015,15 +3015,15 @@
     <row r="19" ht="66" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sky-koi-betta-m4</t>
+          <t xml:space="preserve">sky-koi-betta</t>
         </is>
       </c>
       <c r="B19" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=17abc1d1")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=974c7f77")</f>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta M4</t>
+          <t xml:space="preserve">Sky Koi Betta</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3048,24 +3048,24 @@
     <row r="20" ht="66" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">teal-white-betta</t>
+          <t xml:space="preserve">sky-koi-betta-m4</t>
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=de86fbc9")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=099e8b9d")</f>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+          <t xml:space="preserve">Sky Koi Betta M4</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thân trắng, đuôi xanh ngọc lam, vây bụng cam · màu gốc theo mô hình</t>
+          <t xml:space="preserve">Xanh da trời, đỏ, cam · màu gốc theo mô hình</t>
         </is>
       </c>
       <c r="E20" s="4">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
@@ -3081,31 +3081,64 @@
     <row r="21" ht="66" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">teal-white-betta</t>
+        </is>
+      </c>
+      <c r="B21" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=a25361f1")</f>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thân trắng, đuôi xanh ngọc lam, vây bụng cam · màu gốc theo mô hình</t>
+        </is>
+      </c>
+      <c r="E21" s="4">
+        <v>1300</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solid</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="66" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">yellow-koi-betta</t>
         </is>
       </c>
-      <c r="B21" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=0adb4476")</f>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="B22" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=c8debce1")</f>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Betta Koi Vàng</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Thân vàng cam đốm xanh, đuôi vàng chuyển trắng xanh · màu gốc theo mô hình</t>
         </is>
       </c>
-      <c r="E21" s="4">
+      <c r="E22" s="4">
         <v>1400</v>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Solid</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">1.5</t>
         </is>
@@ -3261,7 +3294,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=1a297ceb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=43252278")</f>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -3302,15 +3335,15 @@
     <row r="5" ht="66" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueBeeBetta</t>
+          <t xml:space="preserve">BlueFlameBetta</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-bee-betta.png?v=f43bfe73")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=9950f4a4")</f>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Ong Xanh</t>
+          <t xml:space="preserve">Blue Flame Betta</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -3347,15 +3380,15 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueFlameBetta</t>
+          <t xml:space="preserve">BluePandaBetta</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=cdd432e5")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=1cbc3e15")</f>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Flame Betta</t>
+          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -3392,15 +3425,15 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BluePandaBetta</t>
+          <t xml:space="preserve">BlueWildBetta</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=36b3bf65")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=e36e243b")</f>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
+          <t xml:space="preserve">Betta Rồng Xanh</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -3437,15 +3470,15 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueWildBetta</t>
+          <t xml:space="preserve">ColorfulBetta</t>
         </is>
       </c>
       <c r="B8" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=680bdef4")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=5cc1541c")</f>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Rồng Xanh</t>
+          <t xml:space="preserve">Colorful Betta</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -3482,15 +3515,15 @@
     <row r="9" ht="66" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ColorfulBetta</t>
+          <t xml:space="preserve">EmeraldRedBetta</t>
         </is>
       </c>
       <c r="B9" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=b244d109")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/emerald-red-betta.png?v=c2d27f6b")</f>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colorful Betta</t>
+          <t xml:space="preserve">Betta Lục Bảo Đỏ</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3531,7 +3564,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=c0b59211")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=ab617dcf")</f>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -3576,7 +3609,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b4f93beb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b85cc880")</f>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -3621,7 +3654,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=e769ef5b")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=798a58a8")</f>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -3666,7 +3699,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=e1ab2904")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=f57fa2a7")</f>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -3703,7 +3736,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=8fa1bfac")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=0a139958")</f>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -3748,7 +3781,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=217c12a3")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=d3f82500")</f>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -3785,11 +3818,11 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=82c21339")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=a66df8df")</f>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plakat Galaxy</t>
+          <t xml:space="preserve">Koi Galaxy Betta</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3818,15 +3851,15 @@
     <row r="17" ht="66" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PurpleRubyBetta</t>
+          <t xml:space="preserve">PurpleMoonBetta</t>
         </is>
       </c>
       <c r="B17" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=dd6ba697")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-moon-betta.png?v=f988dcb3")</f>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
+          <t xml:space="preserve">Betta Trăng Tím</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3863,15 +3896,15 @@
     <row r="18" ht="66" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedSteelBetta</t>
+          <t xml:space="preserve">PurpleRubyBetta</t>
         </is>
       </c>
       <c r="B18" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=b64f1149")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=8b2a77a6")</f>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Steel Betta</t>
+          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -3908,15 +3941,15 @@
     <row r="19" ht="66" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RoyalKoiBetta</t>
+          <t xml:space="preserve">RedSteelBetta</t>
         </is>
       </c>
       <c r="B19" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=e1d369c0")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=e29f7895")</f>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Royal Koi</t>
+          <t xml:space="preserve">Red Steel Betta</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3953,15 +3986,15 @@
     <row r="20" ht="66" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBetta</t>
+          <t xml:space="preserve">RoyalKoiBetta</t>
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=b28bfda2")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=413784be")</f>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta</t>
+          <t xml:space="preserve">Royal Koi</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -3998,15 +4031,15 @@
     <row r="21" ht="66" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBettaM4</t>
+          <t xml:space="preserve">SkyKoiBetta</t>
         </is>
       </c>
       <c r="B21" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=17abc1d1")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=974c7f77")</f>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta M4</t>
+          <t xml:space="preserve">Sky Koi Betta</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -4043,15 +4076,15 @@
     <row r="22" ht="66" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TealWhiteBetta</t>
+          <t xml:space="preserve">SkyKoiBettaM4</t>
         </is>
       </c>
       <c r="B22" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=de86fbc9")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=099e8b9d")</f>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+          <t xml:space="preserve">Sky Koi Betta M4</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -4088,43 +4121,88 @@
     <row r="23" ht="66" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">TealWhiteBetta</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=a25361f1")</f>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MeshyColour</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">YellowKoiBetta</t>
         </is>
       </c>
-      <c r="B23" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=0adb4476")</f>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B24" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=c8debce1")</f>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Betta Koi Vàng</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">MeshyColour</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4296,7 +4374,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=1a297ceb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=43252278")</f>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -4337,15 +4415,15 @@
     <row r="5" ht="66" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueBeeBetta</t>
+          <t xml:space="preserve">BlueFlameBetta</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-bee-betta.png?v=f43bfe73")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=9950f4a4")</f>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Ong Xanh</t>
+          <t xml:space="preserve">Blue Flame Betta</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -4382,15 +4460,15 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueFlameBetta</t>
+          <t xml:space="preserve">BluePandaBetta</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=cdd432e5")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=1cbc3e15")</f>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Flame Betta</t>
+          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -4427,15 +4505,15 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BluePandaBetta</t>
+          <t xml:space="preserve">BlueWildBetta</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=36b3bf65")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=e36e243b")</f>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
+          <t xml:space="preserve">Betta Rồng Xanh</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -4472,15 +4550,15 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueWildBetta</t>
+          <t xml:space="preserve">ColorfulBetta</t>
         </is>
       </c>
       <c r="B8" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=680bdef4")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=5cc1541c")</f>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Rồng Xanh</t>
+          <t xml:space="preserve">Colorful Betta</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -4517,15 +4595,15 @@
     <row r="9" ht="66" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ColorfulBetta</t>
+          <t xml:space="preserve">EmeraldRedBetta</t>
         </is>
       </c>
       <c r="B9" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=b244d109")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/emerald-red-betta.png?v=c2d27f6b")</f>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colorful Betta</t>
+          <t xml:space="preserve">Betta Lục Bảo Đỏ</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -4566,7 +4644,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=c0b59211")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=ab617dcf")</f>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -4611,7 +4689,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b4f93beb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b85cc880")</f>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -4656,7 +4734,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=e769ef5b")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=798a58a8")</f>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -4701,7 +4779,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=e1ab2904")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=f57fa2a7")</f>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -4746,7 +4824,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=8fa1bfac")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=0a139958")</f>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -4791,7 +4869,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=217c12a3")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=d3f82500")</f>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -4836,11 +4914,11 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=82c21339")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=a66df8df")</f>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plakat Galaxy</t>
+          <t xml:space="preserve">Koi Galaxy Betta</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -4877,15 +4955,15 @@
     <row r="17" ht="66" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PurpleRubyBetta</t>
+          <t xml:space="preserve">PurpleMoonBetta</t>
         </is>
       </c>
       <c r="B17" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=dd6ba697")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-moon-betta.png?v=f988dcb3")</f>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
+          <t xml:space="preserve">Betta Trăng Tím</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -4922,15 +5000,15 @@
     <row r="18" ht="66" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedSteelBetta</t>
+          <t xml:space="preserve">PurpleRubyBetta</t>
         </is>
       </c>
       <c r="B18" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=b64f1149")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=8b2a77a6")</f>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Steel Betta</t>
+          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -4967,15 +5045,15 @@
     <row r="19" ht="66" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RoyalKoiBetta</t>
+          <t xml:space="preserve">RedSteelBetta</t>
         </is>
       </c>
       <c r="B19" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=e1d369c0")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=e29f7895")</f>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Royal Koi</t>
+          <t xml:space="preserve">Red Steel Betta</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -5012,15 +5090,15 @@
     <row r="20" ht="66" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBetta</t>
+          <t xml:space="preserve">RoyalKoiBetta</t>
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=b28bfda2")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=413784be")</f>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta</t>
+          <t xml:space="preserve">Royal Koi</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -5057,15 +5135,15 @@
     <row r="21" ht="66" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBettaM4</t>
+          <t xml:space="preserve">SkyKoiBetta</t>
         </is>
       </c>
       <c r="B21" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=17abc1d1")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=974c7f77")</f>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta M4</t>
+          <t xml:space="preserve">Sky Koi Betta</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -5102,15 +5180,15 @@
     <row r="22" ht="66" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TealWhiteBetta</t>
+          <t xml:space="preserve">SkyKoiBettaM4</t>
         </is>
       </c>
       <c r="B22" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=de86fbc9")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=099e8b9d")</f>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+          <t xml:space="preserve">Sky Koi Betta M4</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -5147,43 +5225,88 @@
     <row r="23" ht="66" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">TealWhiteBetta</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=a25361f1")</f>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">YellowKoiBetta</t>
         </is>
       </c>
-      <c r="B23" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=0adb4476")</f>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B24" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=c8debce1")</f>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Betta Koi Vàng</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5213,6 +5336,7 @@
     <col min="15" max="15" width="18" customWidth="1"/>
     <col min="16" max="16" width="18" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5263,40 +5387,45 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">headPatch</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">pigmentDepth</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">scaleRelief</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">scaleEdge</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">scaleEdgeWidth</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">vibrance</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">brightness</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">envReflection</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">baseTexture</t>
         </is>
@@ -5340,16 +5469,16 @@
         <v>0</v>
       </c>
       <c r="K2" s="3">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="L2" s="3">
+      <c r="M2" s="3">
         <v>0</v>
       </c>
-      <c r="M2" s="3">
+      <c r="N2" s="3">
         <v>0.5</v>
-      </c>
-      <c r="N2" s="3">
-        <v>1</v>
       </c>
       <c r="O2" s="3">
         <v>1</v>
@@ -5358,6 +5487,9 @@
         <v>1</v>
       </c>
       <c r="Q2" s="3">
+        <v>1</v>
+      </c>
+      <c r="R2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5395,28 +5527,33 @@
       <c r="I3" s="4">
         <v>0</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K3" s="4">
         <v>0</v>
       </c>
-      <c r="K3" s="4">
+      <c r="L3" s="4">
         <v>0.55</v>
       </c>
-      <c r="L3" s="4">
+      <c r="M3" s="4">
         <v>0</v>
       </c>
-      <c r="M3" s="4">
+      <c r="N3" s="4">
         <v>0.35</v>
       </c>
-      <c r="N3" s="4">
+      <c r="O3" s="4">
         <v>1.3</v>
       </c>
-      <c r="O3" s="4">
+      <c r="P3" s="4">
         <v>1.2</v>
       </c>
-      <c r="P3" s="4">
+      <c r="Q3" s="4">
         <v>0</v>
       </c>
-      <c r="Q3" s="4">
+      <c r="R3" s="4">
         <v>1</v>
       </c>
     </row>
@@ -5427,7 +5564,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=1a297ceb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=43252278")</f>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -5500,6 +5637,11 @@
         </is>
       </c>
       <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5508,15 +5650,15 @@
     <row r="5" ht="66" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueBeeBetta</t>
+          <t xml:space="preserve">BlueFlameBetta</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-bee-betta.png?v=f43bfe73")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=9950f4a4")</f>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Ong Xanh</t>
+          <t xml:space="preserve">Blue Flame Betta</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -5585,6 +5727,11 @@
         </is>
       </c>
       <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5593,15 +5740,15 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueFlameBetta</t>
+          <t xml:space="preserve">BluePandaBetta</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=cdd432e5")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=1cbc3e15")</f>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Flame Betta</t>
+          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -5670,6 +5817,11 @@
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5678,15 +5830,15 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BluePandaBetta</t>
+          <t xml:space="preserve">BlueWildBetta</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=36b3bf65")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=e36e243b")</f>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
+          <t xml:space="preserve">Betta Rồng Xanh</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -5755,6 +5907,11 @@
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5763,15 +5920,15 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueWildBetta</t>
+          <t xml:space="preserve">ColorfulBetta</t>
         </is>
       </c>
       <c r="B8" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=680bdef4")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=5cc1541c")</f>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Rồng Xanh</t>
+          <t xml:space="preserve">Colorful Betta</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -5840,6 +5997,11 @@
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5848,21 +6010,19 @@
     <row r="9" ht="66" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ColorfulBetta</t>
+          <t xml:space="preserve">EmeraldRedBetta</t>
         </is>
       </c>
       <c r="B9" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=b244d109")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/emerald-red-betta.png?v=c2d27f6b")</f>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colorful Betta</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">Betta Lục Bảo Đỏ</t>
+        </is>
+      </c>
+      <c r="D9" s="4">
+        <v>0.25</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
@@ -5874,10 +6034,8 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="G9" s="4">
+        <v>1.4</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -5914,17 +6072,18 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="O9" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="P9" s="4">
+        <v>1.35</v>
       </c>
       <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5937,7 +6096,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=c0b59211")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=ab617dcf")</f>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -6010,6 +6169,11 @@
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6022,7 +6186,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b4f93beb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b85cc880")</f>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -6095,6 +6259,11 @@
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6107,7 +6276,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=e769ef5b")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=798a58a8")</f>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -6182,6 +6351,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="13" ht="66" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -6190,7 +6364,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=e1ab2904")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=f57fa2a7")</f>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -6215,17 +6389,17 @@
       <c r="I13" s="4">
         <v>0</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K13" s="4">
         <v>0</v>
       </c>
-      <c r="K13" s="4">
+      <c r="L13" s="4">
         <v>0.55</v>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
@@ -6247,6 +6421,11 @@
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6259,7 +6438,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=8fa1bfac")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=0a139958")</f>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -6332,6 +6511,11 @@
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6344,7 +6528,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=217c12a3")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=d3f82500")</f>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -6369,17 +6553,17 @@
       <c r="I15" s="4">
         <v>0</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K15" s="4">
         <v>0</v>
       </c>
-      <c r="K15" s="4">
+      <c r="L15" s="4">
         <v>0.55</v>
       </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
@@ -6401,6 +6585,11 @@
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6413,11 +6602,11 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=82c21339")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=a66df8df")</f>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plakat Galaxy</t>
+          <t xml:space="preserve">Koi Galaxy Betta</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -6439,29 +6628,32 @@
         <v>0.04</v>
       </c>
       <c r="J16" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="K16" s="4">
         <v>0.35</v>
       </c>
-      <c r="K16" s="4">
-        <v>0</v>
-      </c>
       <c r="L16" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="M16" s="4">
         <v>1</v>
       </c>
-      <c r="M16" s="4">
+      <c r="N16" s="4">
         <v>0.35</v>
       </c>
-      <c r="N16" s="4">
+      <c r="O16" s="4">
         <v>1.3</v>
       </c>
-      <c r="O16" s="4">
+      <c r="P16" s="4">
         <v>1.12</v>
       </c>
-      <c r="P16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6470,21 +6662,19 @@
     <row r="17" ht="66" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PurpleRubyBetta</t>
+          <t xml:space="preserve">PurpleMoonBetta</t>
         </is>
       </c>
       <c r="B17" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=dd6ba697")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-moon-betta.png?v=f988dcb3")</f>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">Betta Trăng Tím</t>
+        </is>
+      </c>
+      <c r="D17" s="4">
+        <v>0.5</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -6496,10 +6686,8 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="G17" s="4">
+        <v>1.2</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -6546,7 +6734,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q17" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6555,15 +6746,15 @@
     <row r="18" ht="66" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedSteelBetta</t>
+          <t xml:space="preserve">PurpleRubyBetta</t>
         </is>
       </c>
       <c r="B18" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=b64f1149")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=8b2a77a6")</f>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Steel Betta</t>
+          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -6632,6 +6823,11 @@
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6640,15 +6836,15 @@
     <row r="19" ht="66" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RoyalKoiBetta</t>
+          <t xml:space="preserve">RedSteelBetta</t>
         </is>
       </c>
       <c r="B19" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=e1d369c0")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=e29f7895")</f>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Royal Koi</t>
+          <t xml:space="preserve">Red Steel Betta</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -6717,6 +6913,11 @@
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6725,15 +6926,15 @@
     <row r="20" ht="66" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBetta</t>
+          <t xml:space="preserve">RoyalKoiBetta</t>
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=b28bfda2")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=413784be")</f>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta</t>
+          <t xml:space="preserve">Royal Koi</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -6802,6 +7003,11 @@
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6810,15 +7016,15 @@
     <row r="21" ht="66" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBettaM4</t>
+          <t xml:space="preserve">SkyKoiBetta</t>
         </is>
       </c>
       <c r="B21" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=17abc1d1")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=974c7f77")</f>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta M4</t>
+          <t xml:space="preserve">Sky Koi Betta</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -6887,6 +7093,11 @@
         </is>
       </c>
       <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6895,15 +7106,15 @@
     <row r="22" ht="66" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TealWhiteBetta</t>
+          <t xml:space="preserve">SkyKoiBettaM4</t>
         </is>
       </c>
       <c r="B22" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=de86fbc9")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=099e8b9d")</f>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+          <t xml:space="preserve">Sky Koi Betta M4</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -6972,6 +7183,11 @@
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6980,83 +7196,178 @@
     <row r="23" ht="66" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">TealWhiteBetta</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=a25361f1")</f>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">YellowKoiBetta</t>
         </is>
       </c>
-      <c r="B23" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=0adb4476")</f>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B24" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=c8debce1")</f>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Betta Koi Vàng</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="P23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7248,7 +7559,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=1a297ceb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/black-samurai-betta.png?v=43252278")</f>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -7304,15 +7615,15 @@
     <row r="5" ht="66" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueBeeBetta</t>
+          <t xml:space="preserve">BlueFlameBetta</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-bee-betta.png?v=f43bfe73")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=9950f4a4")</f>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Ong Xanh</t>
+          <t xml:space="preserve">Blue Flame Betta</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -7364,15 +7675,15 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueFlameBetta</t>
+          <t xml:space="preserve">BluePandaBetta</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-flame-betta.png?v=cdd432e5")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=1cbc3e15")</f>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue Flame Betta</t>
+          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -7424,15 +7735,15 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BluePandaBetta</t>
+          <t xml:space="preserve">BlueWildBetta</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-panda-betta.png?v=36b3bf65")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=e36e243b")</f>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Gấu Trúc Xanh</t>
+          <t xml:space="preserve">Betta Rồng Xanh</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -7484,15 +7795,15 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BlueWildBetta</t>
+          <t xml:space="preserve">ColorfulBetta</t>
         </is>
       </c>
       <c r="B8" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/blue-wild-betta.png?v=680bdef4")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=5cc1541c")</f>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Rồng Xanh</t>
+          <t xml:space="preserve">Colorful Betta</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -7544,15 +7855,15 @@
     <row r="9" ht="66" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ColorfulBetta</t>
+          <t xml:space="preserve">EmeraldRedBetta</t>
         </is>
       </c>
       <c r="B9" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/colorful-betta.png?v=b244d109")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/emerald-red-betta.png?v=c2d27f6b")</f>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colorful Betta</t>
+          <t xml:space="preserve">Betta Lục Bảo Đỏ</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -7608,7 +7919,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=c0b59211")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/galaxy-betta.png?v=ab617dcf")</f>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -7668,7 +7979,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b4f93beb")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/gold-tiger-betta.png?v=b85cc880")</f>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -7728,7 +8039,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=e769ef5b")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-betta.png?v=798a58a8")</f>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -7788,7 +8099,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=e1ab2904")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/koi-nemo.png?v=f57fa2a7")</f>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -7838,7 +8149,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=8fa1bfac")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/nemo-koi-betta.png?v=0a139958")</f>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -7898,7 +8209,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=217c12a3")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat.png?v=d3f82500")</f>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -7948,11 +8259,11 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=82c21339")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/plakat-galaxy.png?v=a66df8df")</f>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plakat Galaxy</t>
+          <t xml:space="preserve">Koi Galaxy Betta</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -7990,15 +8301,15 @@
     <row r="17" ht="66" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PurpleRubyBetta</t>
+          <t xml:space="preserve">PurpleMoonBetta</t>
         </is>
       </c>
       <c r="B17" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=dd6ba697")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-moon-betta.png?v=f988dcb3")</f>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
+          <t xml:space="preserve">Betta Trăng Tím</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -8050,15 +8361,15 @@
     <row r="18" ht="66" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedSteelBetta</t>
+          <t xml:space="preserve">PurpleRubyBetta</t>
         </is>
       </c>
       <c r="B18" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=b64f1149")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/purple-ruby-betta.png?v=8b2a77a6")</f>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red Steel Betta</t>
+          <t xml:space="preserve">Betta Hồng Ngọc Tím</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -8110,15 +8421,15 @@
     <row r="19" ht="66" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">RoyalKoiBetta</t>
+          <t xml:space="preserve">RedSteelBetta</t>
         </is>
       </c>
       <c r="B19" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=e1d369c0")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/red-steel-betta.png?v=e29f7895")</f>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Royal Koi</t>
+          <t xml:space="preserve">Red Steel Betta</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -8170,15 +8481,15 @@
     <row r="20" ht="66" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBetta</t>
+          <t xml:space="preserve">RoyalKoiBetta</t>
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=b28bfda2")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/royal-koi-betta.png?v=413784be")</f>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta</t>
+          <t xml:space="preserve">Royal Koi</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -8230,15 +8541,15 @@
     <row r="21" ht="66" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SkyKoiBettaM4</t>
+          <t xml:space="preserve">SkyKoiBetta</t>
         </is>
       </c>
       <c r="B21" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=17abc1d1")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta.png?v=974c7f77")</f>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sky Koi Betta M4</t>
+          <t xml:space="preserve">Sky Koi Betta</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -8290,15 +8601,15 @@
     <row r="22" ht="66" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TealWhiteBetta</t>
+          <t xml:space="preserve">SkyKoiBettaM4</t>
         </is>
       </c>
       <c r="B22" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=de86fbc9")</f>
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/sky-koi-betta-m4.png?v=099e8b9d")</f>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+          <t xml:space="preserve">Sky Koi Betta M4</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -8350,58 +8661,118 @@
     <row r="23" ht="66" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">TealWhiteBetta</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/teal-white-betta.png?v=a25361f1")</f>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Betta Trắng Ngọc Lam</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">YellowKoiBetta</t>
         </is>
       </c>
-      <c r="B23" s="3">
-        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=0adb4476")</f>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B24" s="3">
+        <f>IMAGE("https://pub-590970a58ce5426989b3bcd2897271b4.r2.dev/sheet-images/fish/yellow-koi-betta.png?v=c8debce1")</f>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Betta Koi Vàng</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>